<commit_message>
Region pages: KPIs inside the map panel (no duplicate rows), emblem headers; full ship-to address input
- province/district: KPI row and review removed when the map panel shows; chips carry target MTD, sisa, Real/SO
- header of province/district pages shows the regional emblem (assets/logo, fetched by tools/fetch_logos.py)
- gudang upload accepts ALAMAT_LENGKAP; geocoder and site use it instead of the 30-char Rilis address

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsnPeiEdxgJ5FjVjqTRKU9
</commit_message>
<xml_diff>
--- a/admin/template/TEMPLATE_GUDANG.xlsx
+++ b/admin/template/TEMPLATE_GUDANG.xlsx
@@ -424,13 +424,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
@@ -453,15 +453,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>ALAMAT_LENGKAP</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>LAT</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>LON</t>
         </is>
@@ -485,13 +490,18 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Jl. Raya Indarung No. 1, Kel. Indarung, Kec. Lubuk Kilangan, Kota Padang 25237</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>LUBUK KILANGAN</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>-0.9585</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>100.4719</v>
       </c>
     </row>
@@ -506,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -515,33 +525,40 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Isi satu baris per toko/gudang tujuan. Wajib: KODE_TOKO (sama dengan kode toko di Rilis) dan LAT + LON.</t>
+          <t>ALAMAT_LENGKAP: alamat ship-to utuh (jalan, nomor, kelurahan, kecamatan, kota) dari master customer SAP/CSMS. Sistem memakai ini untuk mencari koordinat otomatis; ALAMAT di Rilis terpotong 30 karakter.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LAT/LON dalam derajat desimal, contoh -0.9585 dan 100.4719 (klik kanan titik di Google Maps untuk menyalin).</t>
+          <t>Isi satu baris per toko/gudang tujuan. Wajib: KODE_TOKO (sama dengan kode toko di Rilis) dan LAT + LON.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jika koordinat belum ada, isi KECAMATAN saja: titik ditaruh di pusat kecamatan (perkiraan).</t>
+          <t>LAT/LON dalam derajat desimal, contoh -0.9585 dan 100.4719 (klik kanan titik di Google Maps untuk menyalin).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Boleh upload sebagian; upload berikutnya hanya menambah/menimpa toko yang ada di file.</t>
+          <t>Jika koordinat belum ada, isi KECAMATAN saja: titik ditaruh di pusat kecamatan (perkiraan).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
+        <is>
+          <t>Boleh upload sebagian; upload berikutnya hanya menambah/menimpa toko yang ada di file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>NAMA_TOKO dan ALAMAT hanya untuk membantu pengisian; tidak dipakai sistem.</t>
         </is>

</xml_diff>